<commit_message>
Add title to XLSX document
</commit_message>
<xml_diff>
--- a/tests/anki_addons_dataset/exporter/xlsx/exp_data.xlsx
+++ b/tests/anki_addons_dataset/exporter/xlsx/exp_data.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Addons" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Addons!$A$2:$Q$2</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Addons!$A$3:$Q$3</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,12 +23,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="P2" authorId="0">
+    <comment ref="P3" authorId="0">
       <text>
         <r>
           <rPr>
@@ -39,8 +39,29 @@
           <t xml:space="preserve">Number of GitHub Actions in the repo</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>16</xdr:col>
+                <xdr:colOff>15</xdr:colOff>
+                <xdr:row>1</xdr:row>
+                <xdr:rowOff>10</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>18</xdr:col>
+                <xdr:colOff>18</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>4</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
-    <comment ref="Q2" authorId="0">
+    <comment ref="Q3" authorId="0">
       <text>
         <r>
           <rPr>
@@ -51,13 +72,37 @@
           <t xml:space="preserve">Number of unit-tests in the repo</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>17</xdr:col>
+                <xdr:colOff>15</xdr:colOff>
+                <xdr:row>1</xdr:row>
+                <xdr:rowOff>10</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>19</xdr:col>
+                <xdr:colOff>15</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>4</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
+  <si>
+    <t xml:space="preserve">Anki Addons Dataset</t>
+  </si>
   <si>
     <t xml:space="preserve">Anki Web</t>
   </si>
@@ -141,7 +186,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -163,6 +208,14 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -203,7 +256,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="21">
+  <cellStyleXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -227,11 +280,14 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -240,26 +296,31 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="8">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="15" builtinId="3"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
     <cellStyle name="Currency" xfId="17" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
+    <cellStyle name="Heading 1" xfId="21"/>
     <cellStyle name="*unknown*" xfId="20" builtinId="8"/>
   </cellStyles>
   <dxfs count="2">
@@ -294,34 +355,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -466,7 +527,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:Q4"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.71"/>
@@ -481,148 +542,165 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="10.71"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="O1" s="2"/>
-      <c r="P1" s="2"/>
-      <c r="Q1" s="2"/>
+      <c r="C1" s="0"/>
+      <c r="D1" s="0"/>
+      <c r="E1" s="0"/>
+      <c r="F1" s="0"/>
+      <c r="G1" s="0"/>
+      <c r="J1" s="0"/>
+      <c r="K1" s="0"/>
+      <c r="N1" s="0"/>
+      <c r="O1" s="0"/>
+      <c r="P1" s="0"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>18</v>
-      </c>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
+      <c r="Q2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="P3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q3" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
         <v>1188705668</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" s="1" t="s">
+      <c r="B4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="1" t="n">
+      <c r="D4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="F3" s="1" t="n">
+      <c r="F4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="1" t="n">
+      <c r="G4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H3" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="J3" s="1" t="n">
+      <c r="H4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" s="1" t="n">
         <v>42</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="K4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="L4" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="L3" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="M3" s="1" t="n">
+      <c r="M4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="N3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="O3" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="P3" s="1" t="n">
+      <c r="N4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="P4" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="Q3" s="1" t="n">
+      <c r="Q4" s="1" t="n">
         <v>7</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:Q2"/>
-  <mergeCells count="3">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="L1:Q1"/>
+  <autoFilter ref="A3:Q3"/>
+  <mergeCells count="4">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="L2:Q2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="H3" r:id="rId2" display="link"/>
-    <hyperlink ref="I3" r:id="rId3" display="link"/>
-    <hyperlink ref="L3" r:id="rId4" display="link"/>
+    <hyperlink ref="H4" r:id="rId2" display="link"/>
+    <hyperlink ref="I4" r:id="rId3" display="link"/>
+    <hyperlink ref="L4" r:id="rId4" display="link"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Add "Branches Number" column to XLSX format
</commit_message>
<xml_diff>
--- a/tests/anki_addons_dataset/exporter/xlsx/exp_data.xlsx
+++ b/tests/anki_addons_dataset/exporter/xlsx/exp_data.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Addons" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Addons!$A$3:$Q$3</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Addons!$A$3:$R$3</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -28,7 +28,7 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="P3" authorId="0">
+    <comment ref="Q3" authorId="0">
       <text>
         <r>
           <rPr>
@@ -44,13 +44,13 @@
           <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
-                <xdr:col>16</xdr:col>
+                <xdr:col>17</xdr:col>
                 <xdr:colOff>15</xdr:colOff>
                 <xdr:row>1</xdr:row>
                 <xdr:rowOff>10</xdr:rowOff>
               </xdr:from>
               <xdr:to>
-                <xdr:col>18</xdr:col>
+                <xdr:col>19</xdr:col>
                 <xdr:colOff>18</xdr:colOff>
                 <xdr:row>5</xdr:row>
                 <xdr:rowOff>4</xdr:rowOff>
@@ -61,7 +61,7 @@
         <mc:Fallback/>
       </mc:AlternateContent>
     </comment>
-    <comment ref="Q3" authorId="0">
+    <comment ref="R3" authorId="0">
       <text>
         <r>
           <rPr>
@@ -77,13 +77,13 @@
           <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
-                <xdr:col>17</xdr:col>
+                <xdr:col>18</xdr:col>
                 <xdr:colOff>15</xdr:colOff>
                 <xdr:row>1</xdr:row>
                 <xdr:rowOff>10</xdr:rowOff>
               </xdr:from>
               <xdr:to>
-                <xdr:col>19</xdr:col>
+                <xdr:col>20</xdr:col>
                 <xdr:colOff>15</xdr:colOff>
                 <xdr:row>5</xdr:row>
                 <xdr:rowOff>4</xdr:rowOff>
@@ -99,7 +99,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="29">
   <si>
     <t xml:space="preserve">Anki Addons Dataset</t>
   </si>
@@ -131,6 +131,9 @@
     <t xml:space="preserve">Versions</t>
   </si>
   <si>
+    <t xml:space="preserve">Branches Number</t>
+  </si>
+  <si>
     <t xml:space="preserve">Rating</t>
   </si>
   <si>
@@ -173,7 +176,7 @@
     <t xml:space="preserve">2023-03-15</t>
   </si>
   <si>
-    <t xml:space="preserve">1.0.0</t>
+    <t xml:space="preserve">25.09.2~</t>
   </si>
   <si>
     <t xml:space="preserve">link</t>
@@ -193,7 +196,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -223,12 +226,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -293,14 +290,14 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -321,19 +318,15 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -552,19 +545,20 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="80.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="10.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="6.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="7.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="12.24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="10.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="13.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="50.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="10.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="8.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="6.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="7.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="12.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="10.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="13.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="50.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="10.71"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -580,91 +574,96 @@
         <v>45955</v>
       </c>
       <c r="F1" s="4"/>
-      <c r="H1" s="3" t="s">
+      <c r="G1" s="4"/>
+      <c r="I1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="3"/>
-      <c r="J1" s="5" t="n">
+      <c r="J1" s="3"/>
+      <c r="K1" s="4" t="n">
         <v>46137.6012152778</v>
       </c>
-      <c r="K1" s="5"/>
+      <c r="L1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6" t="s">
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6" t="s">
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6"/>
-      <c r="O2" s="6"/>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="6"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
+      <c r="P2" s="5"/>
+      <c r="Q2" s="5"/>
+      <c r="R2" s="5"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="I3" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="J3" s="7" t="s">
+      <c r="I3" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="K3" s="7" t="s">
+      <c r="J3" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="K3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="L3" s="7" t="s">
+      <c r="L3" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="M3" s="7" t="s">
+      <c r="M3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="N3" s="7" t="s">
+      <c r="N3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="O3" s="7" t="s">
+      <c r="O3" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="P3" s="7" t="s">
+      <c r="P3" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="Q3" s="7" t="s">
+      <c r="Q3" s="6" t="s">
         <v>21</v>
+      </c>
+      <c r="R3" s="6" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -672,70 +671,73 @@
         <v>1188705668</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="1" t="n">
         <v>4</v>
-      </c>
-      <c r="F4" s="1" t="n">
-        <v>0</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H4" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="I4" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="J4" s="1" t="n">
+      <c r="H4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="K4" s="1" t="n">
         <v>42</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="L4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M4" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="L4" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="M4" s="1" t="n">
+      <c r="N4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="N4" s="1" t="s">
-        <v>23</v>
-      </c>
       <c r="O4" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="P4" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q4" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="Q4" s="1" t="n">
+      <c r="R4" s="1" t="n">
         <v>7</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:Q3"/>
+  <autoFilter ref="A3:R3"/>
   <mergeCells count="8">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="E1:F1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="L2:Q2"/>
+    <mergeCell ref="I1:J1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="M2:R2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="H4" r:id="rId2" display="link"/>
-    <hyperlink ref="I4" r:id="rId3" display="link"/>
-    <hyperlink ref="L4" r:id="rId4" display="link"/>
+    <hyperlink ref="I4" r:id="rId2" display="link"/>
+    <hyperlink ref="J4" r:id="rId3" display="link"/>
+    <hyperlink ref="M4" r:id="rId4" display="link"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Detect AI assistance in addon page
</commit_message>
<xml_diff>
--- a/tests/anki_addons_dataset/exporter/xlsx/exp_data.xlsx
+++ b/tests/anki_addons_dataset/exporter/xlsx/exp_data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Addons" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Addons!$A$3:$S$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Addons!$A$3:$T$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -35,7 +35,20 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q3" authorId="0">
+    <comment ref="J3" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>AI tools the author declared building the add-on with, detected in the AnkiWeb page description. Populated even when there is no GitHub repo. Blank = no declaration detected, not proof AI was unused.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="R3" authorId="0">
       <text>
         <r>
           <rPr>
@@ -48,7 +61,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R3" authorId="0">
+    <comment ref="S3" authorId="0">
       <text>
         <r>
           <rPr>
@@ -61,7 +74,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S3" authorId="0">
+    <comment ref="T3" authorId="0">
       <text>
         <r>
           <rPr>
@@ -79,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="33">
   <si>
     <t>Anki Addons Dataset</t>
   </si>
@@ -120,6 +133,9 @@
     <t>Page</t>
   </si>
   <si>
+    <t>Declared AI</t>
+  </si>
+  <si>
     <t>Anki Forum</t>
   </si>
   <si>
@@ -163,6 +179,9 @@
   </si>
   <si>
     <t>link</t>
+  </si>
+  <si>
+    <t>chatgpt</t>
   </si>
   <si>
     <t>2023-09-10</t>
@@ -550,7 +569,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S4"/>
+  <dimension ref="A1:T4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -559,17 +578,19 @@
     <col min="5" max="5" width="8.7109375" customWidth="1"/>
     <col min="6" max="7" width="6.7109375" customWidth="1"/>
     <col min="8" max="8" width="7.7109375" customWidth="1"/>
-    <col min="9" max="11" width="8.7109375" customWidth="1"/>
-    <col min="12" max="12" width="10.7109375" customWidth="1"/>
-    <col min="13" max="14" width="8.7109375" customWidth="1"/>
-    <col min="15" max="15" width="13.7109375" customWidth="1"/>
-    <col min="16" max="16" width="50.7109375" customWidth="1"/>
-    <col min="17" max="17" width="10.7109375" customWidth="1"/>
-    <col min="18" max="18" width="8.7109375" customWidth="1"/>
-    <col min="19" max="19" width="20.7109375" customWidth="1"/>
+    <col min="9" max="9" width="8.7109375" customWidth="1"/>
+    <col min="10" max="10" width="20.7109375" customWidth="1"/>
+    <col min="11" max="12" width="8.7109375" customWidth="1"/>
+    <col min="13" max="13" width="10.7109375" customWidth="1"/>
+    <col min="14" max="15" width="8.7109375" customWidth="1"/>
+    <col min="16" max="16" width="13.7109375" customWidth="1"/>
+    <col min="17" max="17" width="50.7109375" customWidth="1"/>
+    <col min="18" max="18" width="10.7109375" customWidth="1"/>
+    <col min="19" max="19" width="8.7109375" customWidth="1"/>
+    <col min="20" max="20" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19">
+    <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -586,12 +607,13 @@
         <v>2</v>
       </c>
       <c r="J1" s="2"/>
-      <c r="K1" s="3">
+      <c r="K1" s="2"/>
+      <c r="L1" s="3">
         <v>46137.60121527778</v>
       </c>
-      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
     </row>
-    <row r="2" spans="1:19">
+    <row r="2" spans="1:20">
       <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
@@ -603,22 +625,23 @@
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
-      <c r="J2" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="K2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4" t="s">
+        <v>14</v>
+      </c>
       <c r="L2" s="4"/>
-      <c r="M2" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="O2" s="4"/>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
       <c r="R2" s="4"/>
       <c r="S2" s="4"/>
+      <c r="T2" s="4"/>
     </row>
-    <row r="3" spans="1:19">
+    <row r="3" spans="1:20">
       <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
@@ -647,16 +670,16 @@
         <v>12</v>
       </c>
       <c r="J3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K3" s="4" t="s">
         <v>12</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>14</v>
       </c>
       <c r="L3" s="4" t="s">
         <v>15</v>
       </c>
       <c r="M3" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="N3" s="4" t="s">
         <v>18</v>
@@ -676,19 +699,22 @@
       <c r="S3" s="4" t="s">
         <v>23</v>
       </c>
+      <c r="T3" s="4" t="s">
+        <v>24</v>
+      </c>
     </row>
-    <row r="4" spans="1:19">
+    <row r="4" spans="1:20">
       <c r="A4">
         <v>1188705668</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -703,55 +729,58 @@
         <v>0</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="K4">
+        <v>28</v>
+      </c>
+      <c r="J4" t="s">
+        <v>29</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="L4">
         <v>42</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
+        <v>30</v>
+      </c>
+      <c r="N4" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="M4" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="N4">
+      <c r="O4">
         <v>3</v>
       </c>
-      <c r="O4" t="s">
-        <v>25</v>
-      </c>
       <c r="P4" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q4">
+        <v>26</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>31</v>
+      </c>
+      <c r="R4">
         <v>5</v>
       </c>
-      <c r="R4">
+      <c r="S4">
         <v>7</v>
       </c>
-      <c r="S4" t="s">
-        <v>30</v>
+      <c r="T4" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:S3"/>
+  <autoFilter ref="A3:T3"/>
   <mergeCells count="8">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="E1:F1"/>
-    <mergeCell ref="I1:J1"/>
-    <mergeCell ref="K1:L1"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="M2:S2"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="K2:M2"/>
+    <mergeCell ref="N2:T2"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="I4" r:id="rId1"/>
-    <hyperlink ref="J4" r:id="rId2"/>
-    <hyperlink ref="M4" r:id="rId3"/>
+    <hyperlink ref="K4" r:id="rId2"/>
+    <hyperlink ref="N4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId4"/>

</xml_diff>

<commit_message>
Add Language column to XLSX
</commit_message>
<xml_diff>
--- a/tests/anki_addons_dataset/exporter/xlsx/exp_data.xlsx
+++ b/tests/anki_addons_dataset/exporter/xlsx/exp_data.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Addons" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Addons!$A$3:$T$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Addons!$A$3:$U$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -44,11 +44,24 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
+          <t>Human (natural) language of the AnkiWeb add-on description, auto-detected. Blank when the description is empty or too short to classify.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K3" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
           <t>AI tools the author declared building the add-on with, detected in the AnkiWeb page description. Populated even when there is no GitHub repo. Blank = no declaration detected, not proof AI was unused.</t>
         </r>
       </text>
     </comment>
-    <comment ref="R3" authorId="0">
+    <comment ref="S3" authorId="0">
       <text>
         <r>
           <rPr>
@@ -61,7 +74,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S3" authorId="0">
+    <comment ref="T3" authorId="0">
       <text>
         <r>
           <rPr>
@@ -74,7 +87,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T3" authorId="0">
+    <comment ref="U3" authorId="0">
       <text>
         <r>
           <rPr>
@@ -92,7 +105,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="35">
   <si>
     <t>Anki Addons Dataset</t>
   </si>
@@ -133,6 +146,9 @@
     <t>Page</t>
   </si>
   <si>
+    <t>Language</t>
+  </si>
+  <si>
     <t>Declared AI</t>
   </si>
   <si>
@@ -179,6 +195,9 @@
   </si>
   <si>
     <t>link</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>chatgpt</t>
@@ -569,7 +588,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:U4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -579,18 +598,19 @@
     <col min="6" max="7" width="6.7109375" customWidth="1"/>
     <col min="8" max="8" width="7.7109375" customWidth="1"/>
     <col min="9" max="9" width="8.7109375" customWidth="1"/>
-    <col min="10" max="10" width="20.7109375" customWidth="1"/>
-    <col min="11" max="12" width="8.7109375" customWidth="1"/>
-    <col min="13" max="13" width="10.7109375" customWidth="1"/>
-    <col min="14" max="15" width="8.7109375" customWidth="1"/>
-    <col min="16" max="16" width="13.7109375" customWidth="1"/>
-    <col min="17" max="17" width="50.7109375" customWidth="1"/>
-    <col min="18" max="18" width="10.7109375" customWidth="1"/>
-    <col min="19" max="19" width="8.7109375" customWidth="1"/>
-    <col min="20" max="20" width="20.7109375" customWidth="1"/>
+    <col min="10" max="10" width="14.7109375" customWidth="1"/>
+    <col min="11" max="11" width="13.7109375" customWidth="1"/>
+    <col min="12" max="13" width="8.7109375" customWidth="1"/>
+    <col min="14" max="14" width="10.7109375" customWidth="1"/>
+    <col min="15" max="16" width="8.7109375" customWidth="1"/>
+    <col min="17" max="17" width="13.7109375" customWidth="1"/>
+    <col min="18" max="18" width="50.7109375" customWidth="1"/>
+    <col min="19" max="19" width="10.7109375" customWidth="1"/>
+    <col min="20" max="20" width="8.7109375" customWidth="1"/>
+    <col min="21" max="21" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20">
+    <row r="1" spans="1:21">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -608,12 +628,13 @@
       </c>
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
-      <c r="L1" s="3">
+      <c r="L1" s="2"/>
+      <c r="M1" s="3">
         <v>46137.60121527778</v>
       </c>
-      <c r="M1" s="3"/>
+      <c r="N1" s="3"/>
     </row>
-    <row r="2" spans="1:20">
+    <row r="2" spans="1:21">
       <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
@@ -626,22 +647,23 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
-      <c r="K2" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="L2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4" t="s">
+        <v>15</v>
+      </c>
       <c r="M2" s="4"/>
-      <c r="N2" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="O2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
       <c r="R2" s="4"/>
       <c r="S2" s="4"/>
       <c r="T2" s="4"/>
+      <c r="U2" s="4"/>
     </row>
-    <row r="3" spans="1:20">
+    <row r="3" spans="1:21">
       <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
@@ -673,16 +695,16 @@
         <v>13</v>
       </c>
       <c r="K3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="L3" s="4" t="s">
         <v>12</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>15</v>
       </c>
       <c r="M3" s="4" t="s">
         <v>16</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="O3" s="4" t="s">
         <v>19</v>
@@ -702,19 +724,22 @@
       <c r="T3" s="4" t="s">
         <v>24</v>
       </c>
+      <c r="U3" s="4" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="4" spans="1:20">
+    <row r="4" spans="1:21">
       <c r="A4">
         <v>1188705668</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -729,58 +754,61 @@
         <v>0</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J4" t="s">
+        <v>30</v>
+      </c>
+      <c r="K4" t="s">
+        <v>31</v>
+      </c>
+      <c r="L4" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="K4" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="L4">
+      <c r="M4">
         <v>42</v>
       </c>
-      <c r="M4" t="s">
-        <v>30</v>
-      </c>
-      <c r="N4" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="O4">
+      <c r="N4" t="s">
+        <v>32</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="P4">
         <v>3</v>
       </c>
-      <c r="P4" t="s">
-        <v>26</v>
-      </c>
       <c r="Q4" t="s">
-        <v>31</v>
-      </c>
-      <c r="R4">
+        <v>27</v>
+      </c>
+      <c r="R4" t="s">
+        <v>33</v>
+      </c>
+      <c r="S4">
         <v>5</v>
       </c>
-      <c r="S4">
+      <c r="T4">
         <v>7</v>
       </c>
-      <c r="T4" t="s">
-        <v>32</v>
+      <c r="U4" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:T3"/>
+  <autoFilter ref="A3:U3"/>
   <mergeCells count="8">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="E1:F1"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="K2:M2"/>
-    <mergeCell ref="N2:T2"/>
+    <mergeCell ref="I1:L1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="L2:N2"/>
+    <mergeCell ref="O2:U2"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="I4" r:id="rId1"/>
-    <hyperlink ref="K4" r:id="rId2"/>
-    <hyperlink ref="N4" r:id="rId3"/>
+    <hyperlink ref="L4" r:id="rId2"/>
+    <hyperlink ref="O4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId4"/>

</xml_diff>